<commit_message>
Add FXR API schema comparison demos
</commit_message>
<xml_diff>
--- a/Unified_FXR_Starfish_Review.xlsx
+++ b/Unified_FXR_Starfish_Review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Fxr series unification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F486A9DD-782D-4C10-B672-377CDB4E267C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A78FEB-1756-4FBC-A170-C91277B023B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="264">
   <si>
     <t>Unified endpoint review</t>
   </si>
@@ -811,11 +811,6 @@
     <t>Original comparison calls applyImpinjGen2X and scanType FXR-only; Starfish feedback corrects Gen2X support.</t>
   </si>
   <si>
-    <t>Why: FX9600 has applyImpinjGen2X in payload and does not have scanType, documentation needs to be updated for applyImpinjGen2X for FX9600
-Needed: yes
-Fix: No changes required</t>
-  </si>
-  <si>
     <t>Add applyImpinjGen2X to Starfish schema/examples based on its review; do not add scanType. Obtain Kamali’s row 25.</t>
   </si>
   <si>
@@ -861,6 +856,23 @@
   </si>
   <si>
     <t>Retain reported Starfish key case and confirm FXR spelling and capability fields with Kamali.</t>
+  </si>
+  <si>
+    <t>Why: FX9600 has applyImpinjGen2X in payload and does not have scanType, documentation needs to be updated for applyImpinjGen2X for FX9600
+Needed: yes
+Fix: No changes required
+Schema tree - FX9600 (Naveen-confirmed behavior):
+PUT /cloud/start
++-- doNotPersistState (boolean, documented default: true)
+\-- applyImpinjGen2X (boolean; supported, schema update needed)</t>
+  </si>
+  <si>
+    <t>Not provided in the pasted Kamali review.
+Schema tree - FXR60/90 (current schema):
+PUT /cloud/start
++-- doNotPersistState (boolean)
++-- applyImpinjGen2X (boolean)
+\-- scanType (array: ble | rfid)</t>
   </si>
 </sst>
 </file>
@@ -3497,7 +3509,7 @@
       </c>
       <c r="N30" s="11"/>
     </row>
-    <row r="31" spans="1:14" ht="87" customHeight="1">
+    <row r="31" spans="1:14" ht="210" customHeight="1">
       <c r="A31" s="9">
         <v>25</v>
       </c>
@@ -3517,25 +3529,25 @@
         <v>246</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>206</v>
+        <v>263</v>
       </c>
       <c r="I31" s="4" t="s">
         <v>207</v>
       </c>
       <c r="J31" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="K31" s="4" t="s">
         <v>248</v>
-      </c>
-      <c r="K31" s="4" t="s">
-        <v>249</v>
       </c>
       <c r="L31" s="4" t="s">
         <v>210</v>
       </c>
       <c r="M31" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="N31" s="11"/>
     </row>
@@ -3547,7 +3559,7 @@
         <v>13</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>103</v>
@@ -3556,10 +3568,10 @@
         <v>163</v>
       </c>
       <c r="F32" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="G32" s="6" t="s">
         <v>252</v>
-      </c>
-      <c r="G32" s="6" t="s">
-        <v>253</v>
       </c>
       <c r="H32" s="6" t="s">
         <v>206</v>
@@ -3568,16 +3580,16 @@
         <v>207</v>
       </c>
       <c r="J32" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="K32" s="6" t="s">
         <v>254</v>
-      </c>
-      <c r="K32" s="6" t="s">
-        <v>255</v>
       </c>
       <c r="L32" s="6" t="s">
         <v>210</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="N32" s="11"/>
     </row>
@@ -3589,7 +3601,7 @@
         <v>13</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>111</v>
@@ -3598,7 +3610,7 @@
         <v>163</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G33" s="4" t="s">
         <v>242</v>
@@ -3610,14 +3622,14 @@
         <v>207</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="K33" s="4"/>
       <c r="L33" s="4" t="s">
         <v>210</v>
       </c>
       <c r="M33" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="N33" s="11"/>
     </row>
@@ -3629,7 +3641,7 @@
         <v>13</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>103</v>
@@ -3638,7 +3650,7 @@
         <v>163</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G34" s="6" t="s">
         <v>242</v>
@@ -3650,14 +3662,14 @@
         <v>207</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="K34" s="6"/>
       <c r="L34" s="6" t="s">
         <v>210</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="N34" s="11"/>
     </row>

</xml_diff>